<commit_message>
Added an overview page explaining how the spreadsheet works. Plus a bit more data entry since the last check-in.
SVN-Revision: r15
SVN-URL: https://www.cave-registry.org.uk/svn/WookeyCatchment/Swildons
</commit_message>
<xml_diff>
--- a/WISLogbookTranscription/WStantonSurveyBook1.xlsx
+++ b/WISLogbookTranscription/WStantonSurveyBook1.xlsx
@@ -7,17 +7,18 @@
     <workbookView xWindow="480" yWindow="345" windowWidth="22995" windowHeight="9270"/>
   </bookViews>
   <sheets>
-    <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Interpreted Data" sheetId="2" r:id="rId2"/>
-    <sheet name="Survex Formatted" sheetId="3" r:id="rId3"/>
-    <sheet name="Therion Formatted" sheetId="4" r:id="rId4"/>
+    <sheet name="Overview" sheetId="5" r:id="rId1"/>
+    <sheet name="Raw Data" sheetId="1" r:id="rId2"/>
+    <sheet name="Interpreted Data" sheetId="2" r:id="rId3"/>
+    <sheet name="Survex Formatted" sheetId="3" r:id="rId4"/>
+    <sheet name="Therion Formatted" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1781" uniqueCount="868">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1860" uniqueCount="901">
   <si>
     <t>21st July 1951</t>
   </si>
@@ -2621,6 +2622,106 @@
   </si>
   <si>
     <t>280 00</t>
+  </si>
+  <si>
+    <t>176 00</t>
+  </si>
+  <si>
+    <t>325 00</t>
+  </si>
+  <si>
+    <t>145 00</t>
+  </si>
+  <si>
+    <t>157 30</t>
+  </si>
+  <si>
+    <t>283 30</t>
+  </si>
+  <si>
+    <t>103 30</t>
+  </si>
+  <si>
+    <t>140 00</t>
+  </si>
+  <si>
+    <t>139 00</t>
+  </si>
+  <si>
+    <t>074 00</t>
+  </si>
+  <si>
+    <t>6 to foot of slope</t>
+  </si>
+  <si>
+    <t>10 to corner</t>
+  </si>
+  <si>
+    <t>211 00</t>
+  </si>
+  <si>
+    <t>031 00</t>
+  </si>
+  <si>
+    <t>(=PDF p.73-74)</t>
+  </si>
+  <si>
+    <t>(=PDF p.71-72)</t>
+  </si>
+  <si>
+    <t>p. 69-70</t>
+  </si>
+  <si>
+    <t>stalagmite 5</t>
+  </si>
+  <si>
+    <t>3 rocks</t>
+  </si>
+  <si>
+    <t>018 00</t>
+  </si>
+  <si>
+    <t>26 30</t>
+  </si>
+  <si>
+    <t>This spreadsheet was designed for entering and converting the survey data from Willie Stanton's survey notebooks into digital data which could be processed by Survex and Therion cave survey programs. The philosopy for the data entry is to retain as close to the original format of all data as possible at the data entry stage. This enables the data in the spreadsheet to be easily identified with the corresponding data in the original survey notebooks, for cross checking. The spreadsheet is organised into a number of worksheets as described below.</t>
+  </si>
+  <si>
+    <t>Raw Data</t>
+  </si>
+  <si>
+    <t>Interpreted Data</t>
+  </si>
+  <si>
+    <t>Survex Formatted</t>
+  </si>
+  <si>
+    <t>Therion Formatted</t>
+  </si>
+  <si>
+    <t>http://www.mcra.org.uk/logbooks/?dir=Willie%20Stanton%2FSurvey%20Notes</t>
+  </si>
+  <si>
+    <t>The original survey notebooks were obtained as scanned documents in PDF format from the MCRA website:</t>
+  </si>
+  <si>
+    <t>This spreadsheet is stored in the BCA Cave Registry Data Archive:</t>
+  </si>
+  <si>
+    <t>http://cave-registry.org.uk/</t>
+  </si>
+  <si>
+    <t>This sheet is where the raw data entry is being made. The data is entered in columns in as close as possible to the format written in the original notebooks. Page numbers for the original notebooks are specified in addition to the actual page number from the source PDF documents to help indicate the source pages of the data.</t>
+  </si>
+  <si>
+    <t>This sheet is where the data interpretation is done, converting different formatting of numbers into numeric data which the spreadsheet can do operations on. E.g. Angles given in degrees-seconds are converted into decimal degrees. Clino readings for legs where a vertical drop was quoted rather than a clino angle have the clino angle calculated from the other data for the leg. Cells with calculated values using different formulae are coloured differently to help see where data is being derived from (e.g. calculated clino reading as green instead of blue for interpreted angles determined from degrees and minutes). 
+This sheet also contains check-sum calculations to help look for data errors. Vertical and horizontal distances are calculated and compared to the values entered in the Raw Data sheet from the notebooks, and if these differ significantly then the calculated values are coloured red to highlight possible errors in data entry (or in the original source data).</t>
+  </si>
+  <si>
+    <t>This sheet contains data in normal survex format for cutting and pasting into Survex text files for processing. All data is converted into metric decimal units on this worksheet.</t>
+  </si>
+  <si>
+    <t>This sheet contains the data reformatted for Therion survey data files. As much of the original formatting as possible is retained here so that the data in the Therion data files is easier to match to the original survey notebooks as possible.</t>
   </si>
 </sst>
 </file>
@@ -2630,7 +2731,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2667,6 +2768,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2685,10 +2794,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2716,8 +2826,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
@@ -3038,7 +3156,102 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P380"/>
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="118.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15"/>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="120" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="15"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="15"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="15" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="17" t="s">
+        <v>896</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A16" r:id="rId1"/>
+    <hyperlink ref="A19" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P388"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" customWidth="1"/>
@@ -16578,101 +16791,64 @@
       </c>
     </row>
     <row r="334" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A334" t="s">
+      <c r="A334" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="335" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A335" t="s">
         <v>763</v>
       </c>
-      <c r="B334" t="s">
+      <c r="B335" t="s">
         <v>324</v>
       </c>
-      <c r="C334">
+      <c r="C335">
         <v>3</v>
       </c>
-      <c r="D334">
+      <c r="D335">
         <v>3</v>
       </c>
-      <c r="E334">
+      <c r="E335">
         <v>20</v>
       </c>
-      <c r="F334">
+      <c r="F335">
         <v>7</v>
       </c>
-      <c r="G334" t="s">
+      <c r="G335" t="s">
         <v>821</v>
-      </c>
-      <c r="H334" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I334" t="s">
-        <v>831</v>
-      </c>
-      <c r="J334">
-        <v>16.2</v>
-      </c>
-      <c r="K334" t="s">
-        <v>835</v>
-      </c>
-      <c r="M334">
-        <v>14.6</v>
-      </c>
-      <c r="N334">
-        <v>7</v>
-      </c>
-      <c r="O334">
-        <v>358.6</v>
-      </c>
-    </row>
-    <row r="335" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A335" t="str">
-        <f t="shared" ref="A335:A347" si="40">B334</f>
-        <v>EA</v>
-      </c>
-      <c r="C335" s="7" t="str">
-        <f t="shared" ref="C335:F338" si="41">"/"</f>
-        <v>/</v>
-      </c>
-      <c r="D335" s="7" t="str">
-        <f t="shared" si="41"/>
-        <v>/</v>
-      </c>
-      <c r="E335" s="7" t="str">
-        <f t="shared" si="41"/>
-        <v>/</v>
-      </c>
-      <c r="F335" s="7" t="str">
-        <f t="shared" si="41"/>
-        <v>/</v>
-      </c>
-      <c r="G335" s="7" t="s">
-        <v>16</v>
       </c>
       <c r="H335" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I335" t="s">
-        <v>16</v>
-      </c>
-      <c r="J335" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K335" s="7" t="s">
-        <v>16</v>
+        <v>831</v>
+      </c>
+      <c r="J335">
+        <v>16.2</v>
+      </c>
+      <c r="K335" t="s">
+        <v>835</v>
+      </c>
+      <c r="M335">
+        <v>14.6</v>
+      </c>
+      <c r="N335">
+        <v>7</v>
       </c>
       <c r="O335">
-        <v>365.5</v>
-      </c>
-      <c r="P335" t="s">
-        <v>842</v>
+        <v>358.6</v>
       </c>
     </row>
     <row r="336" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A336" t="s">
-        <v>403</v>
-      </c>
-      <c r="B336" t="s">
-        <v>811</v>
+      <c r="A336" t="str">
+        <f t="shared" ref="A336:A348" si="40">B335</f>
+        <v>EA</v>
       </c>
       <c r="C336" s="7" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" ref="C336:F339" si="41">"/"</f>
         <v>/</v>
       </c>
       <c r="D336" s="7" t="str">
@@ -16687,1129 +16863,1137 @@
         <f t="shared" si="41"/>
         <v>/</v>
       </c>
-      <c r="G336" t="s">
-        <v>822</v>
+      <c r="G336" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="H336" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I336" t="s">
+        <v>16</v>
+      </c>
+      <c r="J336" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="K336" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="O336">
+        <v>365.5</v>
+      </c>
+      <c r="P336" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="337" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A337" t="s">
+        <v>403</v>
+      </c>
+      <c r="B337" t="s">
+        <v>811</v>
+      </c>
+      <c r="C337" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>/</v>
+      </c>
+      <c r="D337" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>/</v>
+      </c>
+      <c r="E337" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>/</v>
+      </c>
+      <c r="F337" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>/</v>
+      </c>
+      <c r="G337" t="s">
         <v>822</v>
       </c>
-      <c r="J336">
+      <c r="H337" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I337" t="s">
+        <v>822</v>
+      </c>
+      <c r="J337">
         <v>26.5</v>
       </c>
-      <c r="K336" t="s">
+      <c r="K337" t="s">
         <v>836</v>
       </c>
-      <c r="M336">
+      <c r="M337">
         <v>24.3</v>
       </c>
-      <c r="N336">
+      <c r="N337">
         <v>10.8</v>
       </c>
-      <c r="O336">
+      <c r="O337">
         <v>260.8</v>
       </c>
-      <c r="P336" t="s">
+      <c r="P337" t="s">
         <v>841</v>
-      </c>
-    </row>
-    <row r="337" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A337" t="str">
-        <f t="shared" si="40"/>
-        <v>GH</v>
-      </c>
-      <c r="B337" t="s">
-        <v>812</v>
-      </c>
-      <c r="C337">
-        <v>7</v>
-      </c>
-      <c r="D337">
-        <v>4</v>
-      </c>
-      <c r="E337">
-        <v>6</v>
-      </c>
-      <c r="F337">
-        <v>12</v>
-      </c>
-      <c r="G337" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H337" s="7" t="s">
-        <v>828</v>
-      </c>
-      <c r="I337" t="s">
-        <v>832</v>
-      </c>
-      <c r="J337">
-        <v>20</v>
-      </c>
-      <c r="K337" t="s">
-        <v>837</v>
-      </c>
-      <c r="M337">
-        <v>19.899999999999999</v>
-      </c>
-      <c r="N337">
-        <v>1.2</v>
-      </c>
-      <c r="O337">
-        <v>271.60000000000002</v>
       </c>
     </row>
     <row r="338" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A338" t="str">
         <f t="shared" si="40"/>
-        <v>GI</v>
+        <v>GH</v>
       </c>
       <c r="B338" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="C338">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D338">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E338">
-        <v>8</v>
-      </c>
-      <c r="F338" s="7" t="str">
-        <f t="shared" si="41"/>
-        <v>/</v>
-      </c>
-      <c r="G338" t="s">
-        <v>823</v>
+        <v>6</v>
+      </c>
+      <c r="F338">
+        <v>12</v>
+      </c>
+      <c r="G338" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="H338" s="7" t="s">
-        <v>16</v>
+        <v>828</v>
       </c>
       <c r="I338" t="s">
-        <v>823</v>
+        <v>832</v>
       </c>
       <c r="J338">
-        <v>52.9</v>
+        <v>20</v>
       </c>
       <c r="K338" t="s">
-        <v>182</v>
+        <v>837</v>
       </c>
       <c r="M338">
-        <v>52.2</v>
+        <v>19.899999999999999</v>
       </c>
       <c r="N338">
-        <v>8.6999999999999993</v>
+        <v>1.2</v>
       </c>
       <c r="O338">
-        <v>272.8</v>
+        <v>271.60000000000002</v>
       </c>
     </row>
     <row r="339" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A339" t="str">
         <f t="shared" si="40"/>
-        <v>GJ</v>
+        <v>GI</v>
       </c>
       <c r="B339" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="C339">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D339">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E339">
-        <v>4</v>
-      </c>
-      <c r="F339" t="s">
-        <v>16</v>
-      </c>
-      <c r="G339" s="7" t="s">
-        <v>824</v>
+        <v>8</v>
+      </c>
+      <c r="F339" s="7" t="str">
+        <f t="shared" si="41"/>
+        <v>/</v>
+      </c>
+      <c r="G339" t="s">
+        <v>823</v>
       </c>
       <c r="H339" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I339" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="J339">
-        <v>4</v>
-      </c>
-      <c r="K339" t="str">
-        <f>"-53 30"</f>
-        <v>-53 30</v>
+        <v>52.9</v>
+      </c>
+      <c r="K339" t="s">
+        <v>182</v>
       </c>
       <c r="M339">
-        <v>2.4</v>
+        <v>52.2</v>
       </c>
       <c r="N339">
-        <v>-3.2</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="O339">
-        <v>281.5</v>
+        <v>272.8</v>
       </c>
     </row>
     <row r="340" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A340" t="str">
         <f t="shared" si="40"/>
-        <v>GK</v>
+        <v>GJ</v>
       </c>
       <c r="B340" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="C340">
+        <v>14</v>
+      </c>
+      <c r="D340">
         <v>4</v>
       </c>
-      <c r="D340">
-        <v>0.5</v>
-      </c>
       <c r="E340">
-        <v>2.5</v>
-      </c>
-      <c r="F340">
-        <v>0.3</v>
-      </c>
-      <c r="G340" t="s">
+        <v>4</v>
+      </c>
+      <c r="F340" t="s">
         <v>16</v>
       </c>
+      <c r="G340" s="7" t="s">
+        <v>824</v>
+      </c>
       <c r="H340" s="7" t="s">
-        <v>633</v>
+        <v>16</v>
       </c>
       <c r="I340" t="s">
-        <v>833</v>
+        <v>824</v>
       </c>
       <c r="J340">
-        <v>11.7</v>
-      </c>
-      <c r="K340" t="s">
-        <v>210</v>
+        <v>4</v>
+      </c>
+      <c r="K340" t="str">
+        <f>"-53 30"</f>
+        <v>-53 30</v>
       </c>
       <c r="M340">
-        <v>10.5</v>
+        <v>2.4</v>
       </c>
       <c r="N340">
-        <v>5.0999999999999996</v>
+        <v>-3.2</v>
       </c>
       <c r="O340">
-        <v>278.3</v>
+        <v>281.5</v>
       </c>
     </row>
     <row r="341" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A341" t="str">
         <f t="shared" si="40"/>
-        <v>GL</v>
+        <v>GK</v>
       </c>
       <c r="B341" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="C341">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D341">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E341">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="F341">
-        <v>3</v>
-      </c>
-      <c r="G341" s="7" t="s">
-        <v>769</v>
+        <v>0.3</v>
+      </c>
+      <c r="G341" t="s">
+        <v>16</v>
       </c>
       <c r="H341" s="7" t="s">
-        <v>16</v>
+        <v>633</v>
       </c>
       <c r="I341" t="s">
-        <v>769</v>
+        <v>833</v>
       </c>
       <c r="J341">
-        <v>15.8</v>
+        <v>11.7</v>
       </c>
       <c r="K341" t="s">
         <v>210</v>
       </c>
       <c r="M341">
-        <v>14.2</v>
+        <v>10.5</v>
       </c>
       <c r="N341">
-        <v>6.9</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="O341">
-        <v>283.39999999999998</v>
+        <v>278.3</v>
       </c>
     </row>
     <row r="342" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A342" t="str">
         <f t="shared" si="40"/>
-        <v>GM</v>
+        <v>GL</v>
       </c>
       <c r="B342" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="C342">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D342">
         <v>2</v>
       </c>
       <c r="E342">
-        <v>1</v>
-      </c>
-      <c r="F342" s="7" t="str">
-        <f t="shared" ref="F342" si="42">"/"</f>
-        <v>/</v>
-      </c>
-      <c r="G342" t="s">
+        <v>2</v>
+      </c>
+      <c r="F342">
+        <v>3</v>
+      </c>
+      <c r="G342" s="7" t="s">
+        <v>769</v>
+      </c>
+      <c r="H342" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H342" s="7" t="s">
-        <v>829</v>
-      </c>
       <c r="I342" t="s">
-        <v>834</v>
+        <v>769</v>
       </c>
       <c r="J342">
-        <v>12.8</v>
+        <v>15.8</v>
       </c>
       <c r="K342" t="s">
         <v>210</v>
       </c>
       <c r="M342">
-        <v>11.5</v>
+        <v>14.2</v>
       </c>
       <c r="N342">
-        <v>5.6</v>
+        <v>6.9</v>
       </c>
       <c r="O342">
-        <v>290.3</v>
+        <v>283.39999999999998</v>
       </c>
     </row>
     <row r="343" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A343" t="str">
         <f t="shared" si="40"/>
-        <v>GN</v>
+        <v>GM</v>
       </c>
       <c r="B343" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="C343">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D343">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E343">
-        <v>0.5</v>
-      </c>
-      <c r="F343">
-        <v>6</v>
-      </c>
-      <c r="G343" s="7" t="s">
-        <v>825</v>
+        <v>1</v>
+      </c>
+      <c r="F343" s="7" t="str">
+        <f t="shared" ref="F343" si="42">"/"</f>
+        <v>/</v>
+      </c>
+      <c r="G343" t="s">
+        <v>16</v>
       </c>
       <c r="H343" s="7" t="s">
-        <v>16</v>
+        <v>829</v>
       </c>
       <c r="I343" t="s">
-        <v>825</v>
+        <v>834</v>
       </c>
       <c r="J343">
-        <v>39.9</v>
+        <v>12.8</v>
       </c>
       <c r="K343" t="s">
-        <v>511</v>
+        <v>210</v>
       </c>
       <c r="M343">
-        <v>36.299999999999997</v>
+        <v>11.5</v>
       </c>
       <c r="N343">
-        <v>16.600000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="O343">
-        <v>295.89999999999998</v>
+        <v>290.3</v>
       </c>
     </row>
     <row r="344" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A344" t="str">
         <f t="shared" si="40"/>
-        <v>GO</v>
+        <v>GN</v>
       </c>
       <c r="B344" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="C344">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D344">
-        <v>0.2</v>
+        <v>4</v>
       </c>
       <c r="E344">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="F344">
-        <v>3</v>
-      </c>
-      <c r="G344" t="s">
+        <v>6</v>
+      </c>
+      <c r="G344" s="7" t="s">
+        <v>825</v>
+      </c>
+      <c r="H344" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H344" s="7" t="s">
-        <v>830</v>
-      </c>
       <c r="I344" t="s">
-        <v>831</v>
+        <v>825</v>
       </c>
       <c r="J344">
-        <v>8.9</v>
+        <v>39.9</v>
       </c>
       <c r="K344" t="s">
-        <v>838</v>
+        <v>511</v>
       </c>
       <c r="M344">
-        <v>8.4</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="N344">
-        <v>3</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="O344">
-        <v>312.5</v>
-      </c>
-      <c r="P344" t="s">
-        <v>843</v>
+        <v>295.89999999999998</v>
       </c>
     </row>
     <row r="345" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A345" t="str">
         <f t="shared" si="40"/>
-        <v>GP</v>
+        <v>GO</v>
       </c>
       <c r="B345" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="C345">
         <v>1</v>
       </c>
       <c r="D345">
+        <v>0.2</v>
+      </c>
+      <c r="E345">
+        <v>4</v>
+      </c>
+      <c r="F345">
         <v>3</v>
       </c>
-      <c r="E345">
+      <c r="G345" t="s">
+        <v>16</v>
+      </c>
+      <c r="H345" s="7" t="s">
+        <v>830</v>
+      </c>
+      <c r="I345" t="s">
+        <v>831</v>
+      </c>
+      <c r="J345">
+        <v>8.9</v>
+      </c>
+      <c r="K345" t="s">
+        <v>838</v>
+      </c>
+      <c r="M345">
+        <v>8.4</v>
+      </c>
+      <c r="N345">
         <v>3</v>
       </c>
-      <c r="F345">
-        <v>7</v>
-      </c>
-      <c r="G345" s="7" t="s">
-        <v>826</v>
-      </c>
-      <c r="H345" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I345" t="s">
-        <v>826</v>
-      </c>
-      <c r="J345">
-        <v>27.7</v>
-      </c>
-      <c r="K345" t="s">
-        <v>459</v>
-      </c>
-      <c r="M345">
-        <v>26.8</v>
-      </c>
-      <c r="N345">
-        <v>7.2</v>
-      </c>
       <c r="O345">
-        <v>315.5</v>
+        <v>312.5</v>
       </c>
       <c r="P345" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="346" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A346" t="str">
         <f t="shared" si="40"/>
-        <v>GQ</v>
+        <v>GP</v>
       </c>
       <c r="B346" t="s">
-        <v>757</v>
+        <v>820</v>
       </c>
       <c r="C346">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D346">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E346">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F346">
-        <v>1</v>
-      </c>
-      <c r="G346" t="s">
-        <v>827</v>
+        <v>7</v>
+      </c>
+      <c r="G346" s="7" t="s">
+        <v>826</v>
       </c>
       <c r="H346" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I346" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="J346">
-        <v>9.8000000000000007</v>
+        <v>27.7</v>
       </c>
       <c r="K346" t="s">
-        <v>839</v>
+        <v>459</v>
       </c>
       <c r="M346">
-        <v>9.3000000000000007</v>
+        <v>26.8</v>
       </c>
       <c r="N346">
-        <v>3.3</v>
+        <v>7.2</v>
       </c>
       <c r="O346">
-        <v>322.7</v>
+        <v>315.5</v>
+      </c>
+      <c r="P346" t="s">
+        <v>844</v>
       </c>
     </row>
     <row r="347" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A347" t="str">
         <f t="shared" si="40"/>
-        <v>GR</v>
+        <v>GQ</v>
+      </c>
+      <c r="B347" t="s">
+        <v>757</v>
       </c>
       <c r="C347">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D347">
         <v>2</v>
       </c>
       <c r="E347">
-        <v>1.7</v>
+        <v>3.5</v>
       </c>
       <c r="F347">
-        <v>0.5</v>
-      </c>
-      <c r="G347" s="7" t="s">
-        <v>16</v>
+        <v>1</v>
+      </c>
+      <c r="G347" t="s">
+        <v>827</v>
       </c>
       <c r="H347" s="7" t="s">
         <v>16</v>
       </c>
+      <c r="I347" t="s">
+        <v>827</v>
+      </c>
+      <c r="J347">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="K347" t="s">
+        <v>839</v>
+      </c>
+      <c r="M347">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="N347">
+        <v>3.3</v>
+      </c>
       <c r="O347">
+        <v>322.7</v>
+      </c>
+    </row>
+    <row r="348" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A348" t="str">
+        <f t="shared" si="40"/>
+        <v>GR</v>
+      </c>
+      <c r="C348">
+        <v>1</v>
+      </c>
+      <c r="D348">
+        <v>2</v>
+      </c>
+      <c r="E348">
+        <v>1.7</v>
+      </c>
+      <c r="F348">
+        <v>0.5</v>
+      </c>
+      <c r="G348" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H348" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="O348">
         <v>325.89999999999998</v>
       </c>
-      <c r="P347" t="s">
+      <c r="P348" t="s">
         <v>845</v>
       </c>
     </row>
-    <row r="348" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A348" s="1" t="s">
-        <v>852</v>
-      </c>
-      <c r="P348" t="s">
+    <row r="349" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A349" s="1"/>
+      <c r="B349" s="1"/>
+      <c r="P349" t="s">
         <v>846</v>
       </c>
     </row>
-    <row r="349" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A349" s="1" t="s">
+    <row r="350" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A350" s="1" t="s">
         <v>847</v>
       </c>
-      <c r="C349" t="s">
+      <c r="C350" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="350" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A350">
+    <row r="351" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A351">
         <v>46</v>
       </c>
-      <c r="B350">
+      <c r="B351">
         <v>60</v>
       </c>
-      <c r="C350" s="7" t="str">
-        <f t="shared" ref="C350:H365" si="43">"/"</f>
+      <c r="C351" s="7" t="str">
+        <f t="shared" ref="C351:H365" si="43">"/"</f>
         <v>/</v>
       </c>
-      <c r="D350" s="7" t="str">
+      <c r="D351" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="E350" s="7" t="str">
+      <c r="E351" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="F350" s="7" t="str">
+      <c r="F351" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="G350" s="7" t="str">
+      <c r="G351" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="H350" s="7" t="s">
+      <c r="H351" s="7" t="s">
         <v>849</v>
       </c>
-      <c r="I350" t="s">
+      <c r="I351" t="s">
         <v>850</v>
       </c>
-      <c r="J350">
+      <c r="J351">
         <v>34.299999999999997</v>
       </c>
-      <c r="K350" t="s">
+      <c r="K351" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="351" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A351">
+    <row r="352" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A352">
         <v>60</v>
       </c>
-      <c r="B351">
+      <c r="B352">
         <v>61</v>
       </c>
-      <c r="C351">
+      <c r="C352">
         <v>10</v>
       </c>
-      <c r="D351">
+      <c r="D352">
         <v>8</v>
       </c>
-      <c r="E351">
+      <c r="E352">
         <v>2</v>
       </c>
-      <c r="F351">
+      <c r="F352">
         <v>8</v>
       </c>
-      <c r="G351" t="s">
+      <c r="G352" t="s">
         <v>851</v>
       </c>
-      <c r="H351" s="7" t="str">
+      <c r="H352" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="I351" t="s">
+      <c r="I352" t="s">
         <v>851</v>
       </c>
-      <c r="J351">
+      <c r="J352">
         <v>41.8</v>
       </c>
-      <c r="K351" t="s">
+      <c r="K352" t="s">
         <v>837</v>
       </c>
     </row>
-    <row r="352" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A352">
+    <row r="353" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A353">
         <v>61</v>
       </c>
-      <c r="B352">
+      <c r="B353">
         <v>62</v>
       </c>
-      <c r="C352">
+      <c r="C353">
         <v>8</v>
       </c>
-      <c r="D352">
+      <c r="D353">
         <v>6</v>
       </c>
-      <c r="E352" t="s">
+      <c r="E353" t="s">
         <v>16</v>
       </c>
-      <c r="F352">
+      <c r="F353">
         <v>3</v>
       </c>
-      <c r="G352" s="7" t="str">
+      <c r="G353" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="H352" t="s">
+      <c r="H353" t="s">
         <v>42</v>
       </c>
-      <c r="I352" t="s">
+      <c r="I353" t="s">
         <v>853</v>
       </c>
-      <c r="J352">
+      <c r="J353">
         <v>22.9</v>
       </c>
-      <c r="K352" t="s">
+      <c r="K353" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="353" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A353">
+    <row r="354" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A354">
         <v>62</v>
       </c>
-      <c r="B353">
+      <c r="B354">
         <v>63</v>
       </c>
-      <c r="C353">
+      <c r="C354">
         <v>5</v>
       </c>
-      <c r="D353">
+      <c r="D354">
         <v>7</v>
       </c>
-      <c r="E353">
+      <c r="E354">
         <v>3</v>
       </c>
-      <c r="F353">
+      <c r="F354">
         <v>1</v>
       </c>
-      <c r="G353" t="s">
+      <c r="G354" t="s">
         <v>854</v>
       </c>
-      <c r="H353" s="7" t="str">
+      <c r="H354" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="I353" t="s">
+      <c r="I354" t="s">
         <v>854</v>
       </c>
-      <c r="J353">
+      <c r="J354">
         <v>30.3</v>
       </c>
-      <c r="K353" t="str">
+      <c r="K354" t="str">
         <f>"-5 00"</f>
         <v>-5 00</v>
       </c>
     </row>
-    <row r="354" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A354">
-        <v>63</v>
-      </c>
-      <c r="B354">
-        <v>64</v>
-      </c>
-      <c r="C354">
-        <v>8</v>
-      </c>
-      <c r="D354">
-        <v>2</v>
-      </c>
-      <c r="F354">
-        <v>2</v>
-      </c>
-      <c r="G354" s="7" t="str">
-        <f t="shared" si="43"/>
-        <v>/</v>
-      </c>
-      <c r="H354" t="s">
-        <v>855</v>
-      </c>
-      <c r="I354" t="s">
-        <v>541</v>
-      </c>
-      <c r="J354">
-        <v>12.5</v>
-      </c>
-      <c r="K354" t="s">
-        <v>313</v>
-      </c>
-    </row>
     <row r="355" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A355">
+        <v>63</v>
+      </c>
+      <c r="B355">
         <v>64</v>
       </c>
-      <c r="B355">
-        <v>65</v>
-      </c>
       <c r="C355">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D355">
-        <v>4</v>
-      </c>
-      <c r="E355">
-        <v>3</v>
-      </c>
-      <c r="F355" t="s">
-        <v>16</v>
+        <v>2</v>
+      </c>
+      <c r="F355">
+        <v>2</v>
       </c>
       <c r="G355" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="H355" s="7" t="s">
-        <v>856</v>
+      <c r="H355" t="s">
+        <v>855</v>
       </c>
       <c r="I355" t="s">
-        <v>857</v>
+        <v>541</v>
       </c>
       <c r="J355">
-        <v>15.7</v>
+        <v>12.5</v>
       </c>
       <c r="K355" t="s">
-        <v>837</v>
+        <v>313</v>
       </c>
     </row>
     <row r="356" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A356">
+        <v>64</v>
+      </c>
+      <c r="B356">
         <v>65</v>
       </c>
-      <c r="B356">
-        <v>66</v>
-      </c>
-      <c r="C356" t="s">
-        <v>858</v>
+      <c r="C356">
+        <v>10</v>
       </c>
       <c r="D356">
+        <v>4</v>
+      </c>
+      <c r="E356">
         <v>3</v>
       </c>
-      <c r="E356">
-        <v>2</v>
-      </c>
-      <c r="F356">
-        <v>2</v>
-      </c>
-      <c r="G356" t="s">
-        <v>859</v>
-      </c>
-      <c r="H356" s="7" t="str">
+      <c r="F356" t="s">
+        <v>16</v>
+      </c>
+      <c r="G356" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
+      <c r="H356" s="7" t="s">
+        <v>856</v>
+      </c>
       <c r="I356" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="J356">
-        <v>19.3</v>
+        <v>15.7</v>
       </c>
       <c r="K356" t="s">
-        <v>217</v>
+        <v>837</v>
       </c>
     </row>
     <row r="357" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A357">
+        <v>65</v>
+      </c>
+      <c r="B357">
         <v>66</v>
       </c>
-      <c r="B357">
-        <v>67</v>
-      </c>
-      <c r="C357">
-        <v>6</v>
+      <c r="C357" t="s">
+        <v>858</v>
       </c>
       <c r="D357">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E357">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F357">
-        <v>4</v>
-      </c>
-      <c r="G357" s="7" t="str">
+        <v>2</v>
+      </c>
+      <c r="G357" t="s">
+        <v>859</v>
+      </c>
+      <c r="H357" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="H357" s="7" t="s">
+      <c r="I357" t="s">
+        <v>859</v>
+      </c>
+      <c r="J357">
+        <v>19.3</v>
+      </c>
+      <c r="K357" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="358" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A358">
+        <v>66</v>
+      </c>
+      <c r="B358">
+        <v>67</v>
+      </c>
+      <c r="C358">
+        <v>6</v>
+      </c>
+      <c r="D358">
+        <v>4</v>
+      </c>
+      <c r="E358">
+        <v>3</v>
+      </c>
+      <c r="F358">
+        <v>4</v>
+      </c>
+      <c r="G358" s="7" t="str">
+        <f t="shared" si="43"/>
+        <v>/</v>
+      </c>
+      <c r="H358" s="7" t="s">
         <v>860</v>
       </c>
-      <c r="I357" t="s">
+      <c r="I358" t="s">
         <v>861</v>
       </c>
-      <c r="J357">
+      <c r="J358">
         <v>30.2</v>
       </c>
-      <c r="K357" t="str">
+      <c r="K358" t="str">
         <f>"-1 00"</f>
         <v>-1 00</v>
       </c>
     </row>
-    <row r="358" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A358">
+    <row r="359" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A359">
         <v>67</v>
       </c>
-      <c r="B358">
+      <c r="B359">
         <v>68</v>
       </c>
-      <c r="C358">
+      <c r="C359">
         <v>3</v>
       </c>
-      <c r="D358">
+      <c r="D359">
         <v>2</v>
       </c>
-      <c r="E358">
+      <c r="E359">
         <v>6</v>
       </c>
-      <c r="F358">
+      <c r="F359">
         <v>4</v>
       </c>
-      <c r="G358" t="s">
+      <c r="G359" t="s">
         <v>426</v>
       </c>
-      <c r="H358" s="7" t="str">
+      <c r="H359" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="I358" t="s">
+      <c r="I359" t="s">
         <v>426</v>
       </c>
-      <c r="J358">
+      <c r="J359">
         <v>48.9</v>
       </c>
-      <c r="K358" t="str">
+      <c r="K359" t="str">
         <f>"-4 00"</f>
         <v>-4 00</v>
       </c>
     </row>
-    <row r="359" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A359">
+    <row r="360" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A360">
         <v>68</v>
       </c>
-      <c r="B359">
+      <c r="B360">
         <v>69</v>
       </c>
-      <c r="C359">
+      <c r="C360">
         <v>3</v>
       </c>
-      <c r="D359">
+      <c r="D360">
         <v>3</v>
       </c>
-      <c r="E359">
+      <c r="E360">
         <v>1</v>
       </c>
-      <c r="F359" t="s">
+      <c r="F360" t="s">
         <v>16</v>
       </c>
-      <c r="G359" s="7" t="str">
+      <c r="G360" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="H359" s="7" t="s">
+      <c r="H360" s="7" t="s">
         <v>862</v>
       </c>
-      <c r="I359" t="s">
+      <c r="I360" t="s">
         <v>863</v>
       </c>
-      <c r="J359">
+      <c r="J360">
         <v>14.8</v>
       </c>
-      <c r="K359" t="s">
+      <c r="K360" t="s">
         <v>656</v>
       </c>
     </row>
-    <row r="360" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A360">
+    <row r="361" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A361">
         <v>69</v>
       </c>
-      <c r="B360">
+      <c r="B361">
         <v>70</v>
       </c>
-      <c r="C360">
+      <c r="C361">
         <v>6</v>
       </c>
-      <c r="D360">
+      <c r="D361">
         <v>3</v>
       </c>
-      <c r="E360">
+      <c r="E361">
         <v>3</v>
       </c>
-      <c r="F360">
+      <c r="F361">
         <v>3</v>
       </c>
-      <c r="G360" t="s">
+      <c r="G361" t="s">
         <v>864</v>
       </c>
-      <c r="H360" s="7" t="str">
+      <c r="H361" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="I360" t="s">
+      <c r="I361" t="s">
         <v>864</v>
       </c>
-      <c r="J360">
+      <c r="J361">
         <v>21</v>
       </c>
-      <c r="K360" t="str">
+      <c r="K361" t="str">
         <f>"-6 30"</f>
         <v>-6 30</v>
       </c>
     </row>
-    <row r="361" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A361">
+    <row r="362" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A362">
         <v>70</v>
       </c>
-      <c r="B361">
+      <c r="B362">
         <v>71</v>
       </c>
-      <c r="C361">
+      <c r="C362">
         <v>3</v>
       </c>
-      <c r="D361">
+      <c r="D362">
         <v>1</v>
       </c>
-      <c r="E361">
+      <c r="E362">
         <v>3</v>
       </c>
-      <c r="F361" s="7" t="str">
+      <c r="F362" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="G361" s="7" t="str">
+      <c r="G362" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="H361" t="s">
+      <c r="H362" t="s">
         <v>363</v>
       </c>
-      <c r="I361" t="s">
+      <c r="I362" t="s">
         <v>356</v>
       </c>
-      <c r="J361">
+      <c r="J362">
         <v>36.799999999999997</v>
       </c>
-      <c r="K361" t="s">
+      <c r="K362" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="362" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A362">
+    <row r="363" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A363">
         <v>71</v>
       </c>
-      <c r="B362">
+      <c r="B363">
         <v>72</v>
       </c>
-      <c r="C362">
+      <c r="C363">
         <v>4</v>
       </c>
-      <c r="D362">
+      <c r="D363">
         <v>3</v>
       </c>
-      <c r="E362" t="s">
+      <c r="E363" t="s">
         <v>865</v>
       </c>
-      <c r="F362">
+      <c r="F363">
         <v>5</v>
       </c>
-      <c r="G362" t="s">
+      <c r="G363" t="s">
         <v>866</v>
       </c>
-      <c r="H362" s="7" t="str">
+      <c r="H363" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="I362" t="s">
+      <c r="I363" t="s">
         <v>866</v>
       </c>
-      <c r="J362">
+      <c r="J363">
         <v>38.200000000000003</v>
       </c>
-      <c r="K362" t="s">
+      <c r="K363" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="363" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A363">
+    <row r="364" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A364">
         <v>72</v>
       </c>
-      <c r="B363">
+      <c r="B364">
         <v>73</v>
       </c>
-      <c r="C363">
+      <c r="C364">
         <v>8</v>
       </c>
-      <c r="D363">
+      <c r="D364">
         <v>4</v>
       </c>
-      <c r="E363">
+      <c r="E364">
         <v>3</v>
       </c>
-      <c r="F363" t="s">
+      <c r="F364" t="s">
         <v>16</v>
       </c>
-      <c r="G363" s="7" t="str">
+      <c r="G364" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="H363" t="s">
+      <c r="H364" t="s">
         <v>516</v>
       </c>
-      <c r="I363" t="s">
+      <c r="I364" t="s">
         <v>515</v>
       </c>
-      <c r="J363">
+      <c r="J364">
         <v>11.9</v>
       </c>
-      <c r="K363" t="str">
+      <c r="K364" t="str">
         <f>"-10 00"</f>
         <v>-10 00</v>
       </c>
     </row>
-    <row r="364" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A364">
+    <row r="365" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A365">
         <v>73</v>
       </c>
-      <c r="B364">
+      <c r="B365">
         <v>74</v>
       </c>
-      <c r="C364">
+      <c r="C365">
         <v>15</v>
       </c>
-      <c r="D364">
+      <c r="D365">
         <v>2</v>
       </c>
-      <c r="E364">
+      <c r="E365">
         <v>3</v>
       </c>
-      <c r="F364">
+      <c r="F365">
         <v>2</v>
       </c>
-      <c r="G364" t="s">
+      <c r="G365" t="s">
         <v>623</v>
       </c>
-      <c r="H364" s="7" t="str">
+      <c r="H365" s="7" t="str">
         <f t="shared" si="43"/>
         <v>/</v>
       </c>
-      <c r="I364" t="s">
+      <c r="I365" t="s">
         <v>623</v>
       </c>
-      <c r="J364">
+      <c r="J365">
         <v>34.200000000000003</v>
       </c>
-      <c r="K364" t="str">
+      <c r="K365" t="str">
         <f>"-1 30"</f>
         <v>-1 30</v>
       </c>
     </row>
-    <row r="365" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A365">
-        <v>74</v>
-      </c>
-      <c r="B365">
-        <v>75</v>
-      </c>
-      <c r="C365">
-        <v>4</v>
-      </c>
-      <c r="D365" t="s">
-        <v>16</v>
-      </c>
-      <c r="E365">
-        <v>3</v>
-      </c>
-      <c r="F365" t="s">
-        <v>865</v>
-      </c>
-      <c r="G365" s="7" t="str">
-        <f t="shared" ref="G365:H379" si="44">"/"</f>
-        <v>/</v>
-      </c>
-      <c r="H365" t="s">
-        <v>867</v>
-      </c>
-      <c r="I365" t="s">
-        <v>548</v>
-      </c>
-      <c r="J365">
-        <v>9.1</v>
-      </c>
-      <c r="K365" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="366" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A366">
+        <v>74</v>
+      </c>
+      <c r="B366">
         <v>75</v>
-      </c>
-      <c r="B366">
-        <v>76</v>
       </c>
       <c r="C366">
         <v>4</v>
@@ -17818,186 +18002,775 @@
         <v>16</v>
       </c>
       <c r="E366">
+        <v>3</v>
+      </c>
+      <c r="F366" t="s">
+        <v>865</v>
+      </c>
+      <c r="G366" s="7" t="str">
+        <f t="shared" ref="F366:H385" si="44">"/"</f>
+        <v>/</v>
+      </c>
+      <c r="H366" t="s">
+        <v>867</v>
+      </c>
+      <c r="I366" t="s">
+        <v>548</v>
+      </c>
+      <c r="J366">
+        <v>9.1</v>
+      </c>
+      <c r="K366" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="367" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A367">
+        <v>75</v>
+      </c>
+      <c r="B367">
+        <v>76</v>
+      </c>
+      <c r="C367">
+        <v>4</v>
+      </c>
+      <c r="D367" t="s">
+        <v>16</v>
+      </c>
+      <c r="E367">
         <v>1</v>
       </c>
-      <c r="F366">
+      <c r="F367">
         <v>2</v>
       </c>
-      <c r="G366" s="7" t="str">
+      <c r="G367" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-      <c r="H366" s="7" t="s">
+      <c r="H367" s="7" t="s">
         <v>721</v>
       </c>
-      <c r="I366" t="s">
+      <c r="I367" t="s">
         <v>729</v>
       </c>
-      <c r="J366">
+      <c r="J367">
         <v>40.700000000000003</v>
       </c>
-      <c r="K366" t="s">
+      <c r="K367" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="367" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A367">
+    <row r="368" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A368">
         <v>76</v>
       </c>
-      <c r="B367">
+      <c r="B368">
         <v>77</v>
       </c>
-      <c r="H367" s="7" t="str">
+      <c r="C368">
+        <v>10</v>
+      </c>
+      <c r="D368">
+        <v>2</v>
+      </c>
+      <c r="E368">
+        <v>1</v>
+      </c>
+      <c r="F368">
+        <v>2</v>
+      </c>
+      <c r="G368" t="s">
+        <v>244</v>
+      </c>
+      <c r="H368" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="368" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A368">
+      <c r="I368" t="s">
+        <v>244</v>
+      </c>
+      <c r="J368">
+        <v>17.5</v>
+      </c>
+      <c r="K368" t="str">
+        <f>"-1 30"</f>
+        <v>-1 30</v>
+      </c>
+    </row>
+    <row r="369" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A369">
         <v>77</v>
       </c>
-      <c r="B368">
+      <c r="B369">
         <v>78</v>
       </c>
-      <c r="G368" s="7" t="str">
+      <c r="C369">
+        <v>2</v>
+      </c>
+      <c r="D369" t="s">
+        <v>16</v>
+      </c>
+      <c r="E369">
+        <v>2</v>
+      </c>
+      <c r="F369">
+        <v>2</v>
+      </c>
+      <c r="G369" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="369" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A369">
+      <c r="H369" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="I369" t="s">
+        <v>290</v>
+      </c>
+      <c r="J369">
+        <v>7.6</v>
+      </c>
+      <c r="K369" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="370" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A370">
         <v>78</v>
       </c>
-      <c r="B369">
+      <c r="B370">
         <v>79</v>
       </c>
-      <c r="H369" s="7" t="str">
+      <c r="C370">
+        <v>10</v>
+      </c>
+      <c r="D370">
+        <v>3</v>
+      </c>
+      <c r="E370">
+        <v>3</v>
+      </c>
+      <c r="F370">
+        <v>4</v>
+      </c>
+      <c r="G370" t="s">
+        <v>868</v>
+      </c>
+      <c r="H370" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="370" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A370">
+      <c r="I370" t="s">
+        <v>868</v>
+      </c>
+      <c r="J370">
+        <v>35</v>
+      </c>
+      <c r="K370" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="371" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A371">
         <v>79</v>
       </c>
-      <c r="B370">
+      <c r="B371">
         <v>80</v>
       </c>
-      <c r="G370" s="7" t="str">
+      <c r="C371">
+        <v>10</v>
+      </c>
+      <c r="D371">
+        <v>3</v>
+      </c>
+      <c r="E371">
+        <v>4</v>
+      </c>
+      <c r="F371">
+        <v>4</v>
+      </c>
+      <c r="G371" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="371" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A371">
+      <c r="H371" s="7" t="s">
+        <v>869</v>
+      </c>
+      <c r="I371" t="s">
+        <v>870</v>
+      </c>
+      <c r="J371">
+        <v>45.7</v>
+      </c>
+      <c r="K371" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="372" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A372">
         <v>80</v>
       </c>
-      <c r="B371">
+      <c r="B372">
         <v>81</v>
       </c>
-      <c r="H371" s="7" t="str">
+      <c r="C372">
+        <v>10</v>
+      </c>
+      <c r="D372">
+        <v>3</v>
+      </c>
+      <c r="E372">
+        <v>5</v>
+      </c>
+      <c r="F372">
+        <v>2</v>
+      </c>
+      <c r="G372" t="s">
+        <v>871</v>
+      </c>
+      <c r="H372" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="372" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A372">
+      <c r="I372" t="s">
+        <v>871</v>
+      </c>
+      <c r="J372">
+        <v>27.2</v>
+      </c>
+      <c r="K372" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="373" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A373">
         <v>81</v>
       </c>
-      <c r="B372">
+      <c r="B373">
         <v>82</v>
       </c>
-      <c r="G372" s="7" t="str">
+      <c r="C373">
+        <v>5</v>
+      </c>
+      <c r="D373" t="s">
+        <v>16</v>
+      </c>
+      <c r="E373">
+        <v>7</v>
+      </c>
+      <c r="F373">
+        <v>8</v>
+      </c>
+      <c r="G373" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="373" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A373">
+      <c r="H373" t="s">
+        <v>872</v>
+      </c>
+      <c r="I373" t="s">
+        <v>873</v>
+      </c>
+      <c r="J373">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="K373" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="374" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A374">
         <v>82</v>
       </c>
-      <c r="B373">
+      <c r="B374">
         <v>83</v>
       </c>
-      <c r="H373" s="7" t="str">
+      <c r="C374">
+        <v>2</v>
+      </c>
+      <c r="D374">
+        <v>2</v>
+      </c>
+      <c r="E374">
+        <v>8</v>
+      </c>
+      <c r="F374">
+        <v>6</v>
+      </c>
+      <c r="G374" t="s">
+        <v>874</v>
+      </c>
+      <c r="H374" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="374" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A374">
+      <c r="I374" t="s">
+        <v>874</v>
+      </c>
+      <c r="J374">
+        <v>39.700000000000003</v>
+      </c>
+      <c r="K374" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="375" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A375">
         <v>83</v>
       </c>
-      <c r="B374">
+      <c r="B375">
         <v>84</v>
       </c>
-      <c r="G374" s="7" t="str">
+      <c r="C375">
+        <v>3</v>
+      </c>
+      <c r="D375">
+        <v>1</v>
+      </c>
+      <c r="E375">
+        <v>5</v>
+      </c>
+      <c r="F375">
+        <v>5</v>
+      </c>
+      <c r="G375" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="375" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A375">
+      <c r="H375" t="s">
+        <v>715</v>
+      </c>
+      <c r="I375" t="s">
+        <v>875</v>
+      </c>
+      <c r="J375">
+        <v>35.5</v>
+      </c>
+      <c r="K375" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="376" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A376">
         <v>84</v>
       </c>
-      <c r="B375">
+      <c r="B376">
         <v>85</v>
       </c>
-      <c r="H375" s="7" t="str">
-        <f t="shared" ref="H375:H378" si="45">"/"</f>
+      <c r="C376">
+        <v>1</v>
+      </c>
+      <c r="D376">
+        <v>3</v>
+      </c>
+      <c r="E376">
+        <v>6</v>
+      </c>
+      <c r="F376">
+        <v>3</v>
+      </c>
+      <c r="G376" t="s">
+        <v>876</v>
+      </c>
+      <c r="H376" s="7" t="str">
+        <f t="shared" ref="H376" si="45">"/"</f>
         <v>/</v>
       </c>
-    </row>
-    <row r="376" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A376">
+      <c r="I376" t="s">
+        <v>876</v>
+      </c>
+      <c r="J376">
+        <v>29.1</v>
+      </c>
+      <c r="K376" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="377" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A377">
         <v>85</v>
       </c>
-      <c r="B376">
+      <c r="B377">
         <v>86</v>
       </c>
-      <c r="G376" s="7" t="str">
+      <c r="C377">
+        <v>3</v>
+      </c>
+      <c r="D377" t="s">
+        <v>877</v>
+      </c>
+      <c r="E377">
+        <v>5</v>
+      </c>
+      <c r="F377" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="377" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A377">
-        <v>86</v>
-      </c>
-      <c r="B377">
-        <v>87</v>
-      </c>
-      <c r="H377" s="7" t="str">
+      <c r="G377" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="378" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H377" t="s">
+        <v>773</v>
+      </c>
+      <c r="I377" t="s">
+        <v>621</v>
+      </c>
+      <c r="J377">
+        <v>25.3</v>
+      </c>
+      <c r="K377" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="378" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A378">
+        <v>86</v>
+      </c>
+      <c r="B378">
         <v>87</v>
       </c>
-      <c r="B378">
-        <v>88</v>
-      </c>
-      <c r="G378" s="7" t="str">
+      <c r="C378">
+        <v>3</v>
+      </c>
+      <c r="D378">
+        <v>2</v>
+      </c>
+      <c r="E378">
+        <v>7</v>
+      </c>
+      <c r="F378">
+        <v>3</v>
+      </c>
+      <c r="G378" t="s">
+        <v>652</v>
+      </c>
+      <c r="H378" s="7" t="str">
         <f t="shared" si="44"/>
         <v>/</v>
       </c>
-    </row>
-    <row r="379" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I378" t="s">
+        <v>652</v>
+      </c>
+      <c r="J378">
+        <v>23.1</v>
+      </c>
+      <c r="K378" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="379" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A379">
+        <v>87</v>
+      </c>
+      <c r="B379">
         <v>88</v>
       </c>
-      <c r="B379">
+      <c r="C379">
+        <v>15</v>
+      </c>
+      <c r="D379">
+        <v>6</v>
+      </c>
+      <c r="E379">
+        <v>15</v>
+      </c>
+      <c r="F379" t="s">
+        <v>878</v>
+      </c>
+      <c r="G379" s="7" t="str">
+        <f t="shared" si="44"/>
+        <v>/</v>
+      </c>
+      <c r="H379" t="s">
+        <v>733</v>
+      </c>
+      <c r="I379" t="s">
+        <v>724</v>
+      </c>
+      <c r="J379">
+        <v>51.3</v>
+      </c>
+      <c r="K379" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="380" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A380">
+        <v>88</v>
+      </c>
+      <c r="B380">
         <v>89</v>
       </c>
-    </row>
-    <row r="380" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A380">
+      <c r="C380">
+        <v>22</v>
+      </c>
+      <c r="D380">
+        <v>3</v>
+      </c>
+      <c r="E380">
+        <v>4</v>
+      </c>
+      <c r="F380">
+        <v>5</v>
+      </c>
+      <c r="G380" t="s">
+        <v>229</v>
+      </c>
+      <c r="H380" s="7" t="str">
+        <f t="shared" si="44"/>
+        <v>/</v>
+      </c>
+      <c r="I380" t="s">
+        <v>229</v>
+      </c>
+      <c r="J380">
+        <v>16.5</v>
+      </c>
+      <c r="K380" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="381" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A381">
         <v>89</v>
       </c>
-      <c r="B380">
+      <c r="B381">
         <v>90</v>
+      </c>
+      <c r="C381">
+        <v>24</v>
+      </c>
+      <c r="D381">
+        <v>6</v>
+      </c>
+      <c r="E381">
+        <v>1</v>
+      </c>
+      <c r="F381">
+        <v>4</v>
+      </c>
+      <c r="G381" s="7" t="str">
+        <f t="shared" si="44"/>
+        <v>/</v>
+      </c>
+      <c r="H381" t="s">
+        <v>879</v>
+      </c>
+      <c r="I381" t="s">
+        <v>880</v>
+      </c>
+      <c r="J381">
+        <v>26.4</v>
+      </c>
+      <c r="K381" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="382" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A382" s="1" t="s">
+        <v>852</v>
+      </c>
+      <c r="B382" s="1" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="383" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A383">
+        <v>90</v>
+      </c>
+      <c r="B383">
+        <v>91</v>
+      </c>
+      <c r="C383">
+        <v>15</v>
+      </c>
+      <c r="D383">
+        <v>4</v>
+      </c>
+      <c r="E383">
+        <v>3</v>
+      </c>
+      <c r="F383">
+        <v>3</v>
+      </c>
+      <c r="G383" t="s">
+        <v>425</v>
+      </c>
+      <c r="H383" s="7" t="str">
+        <f t="shared" si="44"/>
+        <v>/</v>
+      </c>
+      <c r="I383" t="s">
+        <v>425</v>
+      </c>
+      <c r="J383">
+        <v>49</v>
+      </c>
+      <c r="K383" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="384" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A384">
+        <v>91</v>
+      </c>
+      <c r="B384">
+        <v>92</v>
+      </c>
+      <c r="C384">
+        <v>25</v>
+      </c>
+      <c r="D384" t="s">
+        <v>885</v>
+      </c>
+      <c r="E384" t="s">
+        <v>16</v>
+      </c>
+      <c r="F384">
+        <v>5</v>
+      </c>
+      <c r="G384" s="7" t="str">
+        <f t="shared" si="44"/>
+        <v>/</v>
+      </c>
+      <c r="H384" t="s">
+        <v>777</v>
+      </c>
+      <c r="I384" t="s">
+        <v>767</v>
+      </c>
+      <c r="J384">
+        <v>35.799999999999997</v>
+      </c>
+      <c r="K384" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="385" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A385">
+        <v>92</v>
+      </c>
+      <c r="B385">
+        <v>93</v>
+      </c>
+      <c r="C385">
+        <v>20</v>
+      </c>
+      <c r="D385">
+        <v>4</v>
+      </c>
+      <c r="E385">
+        <v>8</v>
+      </c>
+      <c r="F385">
+        <v>6</v>
+      </c>
+      <c r="G385" t="s">
+        <v>886</v>
+      </c>
+      <c r="H385" s="7" t="str">
+        <f t="shared" si="44"/>
+        <v>/</v>
+      </c>
+      <c r="I385" t="s">
+        <v>886</v>
+      </c>
+      <c r="J385">
+        <v>48.2</v>
+      </c>
+      <c r="K385" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="386" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A386">
+        <v>93</v>
+      </c>
+      <c r="B386">
+        <v>94</v>
+      </c>
+      <c r="C386">
+        <v>8</v>
+      </c>
+      <c r="D386">
+        <v>7</v>
+      </c>
+      <c r="E386">
+        <v>5</v>
+      </c>
+      <c r="F386">
+        <v>2</v>
+      </c>
+      <c r="G386" s="7" t="str">
+        <f t="shared" ref="G386:H387" si="46">"/"</f>
+        <v>/</v>
+      </c>
+      <c r="H386" t="s">
+        <v>879</v>
+      </c>
+      <c r="I386" t="s">
+        <v>880</v>
+      </c>
+      <c r="J386">
+        <v>18.5</v>
+      </c>
+      <c r="K386" t="str">
+        <f>"-9 00"</f>
+        <v>-9 00</v>
+      </c>
+    </row>
+    <row r="387" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A387">
+        <v>94</v>
+      </c>
+      <c r="B387">
+        <v>95</v>
+      </c>
+      <c r="C387" t="s">
+        <v>884</v>
+      </c>
+      <c r="D387">
+        <v>3</v>
+      </c>
+      <c r="E387">
+        <v>3</v>
+      </c>
+      <c r="F387">
+        <v>1</v>
+      </c>
+      <c r="G387" t="s">
+        <v>646</v>
+      </c>
+      <c r="H387" s="7" t="str">
+        <f t="shared" si="46"/>
+        <v>/</v>
+      </c>
+      <c r="I387" t="s">
+        <v>646</v>
+      </c>
+      <c r="J387">
+        <v>26</v>
+      </c>
+      <c r="K387" t="str">
+        <f>"-4 30"</f>
+        <v>-4 30</v>
+      </c>
+    </row>
+    <row r="388" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A388">
+        <v>95</v>
+      </c>
+      <c r="C388">
+        <v>10</v>
+      </c>
+      <c r="D388" t="s">
+        <v>16</v>
+      </c>
+      <c r="E388" t="s">
+        <v>16</v>
+      </c>
+      <c r="F388">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -18009,7 +18782,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Y281"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -44066,7 +44839,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E280"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -49929,7 +50702,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P327"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>